<commit_message>
sample table update + readme update
</commit_message>
<xml_diff>
--- a/excels/EnumTypes/SampleType.xlsx
+++ b/excels/EnumTypes/SampleType.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuankun.h\Desktop\GameDataConfigTool\excels\EnumTypes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\GameDataConfigTool\excels\EnumTypes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F378D9AA-0E54-48DC-8269-1682EB0FF91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FB2BE5D-395C-4823-870B-8E78B8D4BAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3195" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Name</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>法师</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>未知</t>
   </si>
 </sst>
 </file>
@@ -363,7 +369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
@@ -382,23 +388,34 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>